<commit_message>
feature change: the build_todo only creates steps to write content
</commit_message>
<xml_diff>
--- a/example_prompts.xlsx
+++ b/example_prompts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\KHAN\Python\DocBuilder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{667DD536-E304-481B-BD39-76CFDD47AA88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8431269C-6FA8-448F-94F5-717C2FDD7107}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{C5257242-E22F-4E00-B9FA-96C14573D14B}"/>
   </bookViews>
@@ -47,20 +47,10 @@
     <t>We are planning an Agentic AI project that builds word documents based on plain human prompts. The app will take user prompt, this prompt will be sent to LLMs that will generate the task (for subsequent LLM) and finally create the word doc. Please help us create a word doc for this</t>
   </si>
   <si>
-    <t>&lt;write_paragraph&gt;
-# Agentic AI Project Plan
-## Introduction
-The Agentic AI project aims to create a system that generates word documents based on plain human prompts. This will be achieved by leveraging the capabilities of Large Language Models (LLMs) to process user input and produce high-quality documents.
-## System Architecture
-&lt;stop_write_paragraph&gt;
-&lt;write_ordered_list&gt;
-1. **User Prompt**: The user will provide a plain text prompt that will be used as input for the system.
-2. **LLM 1: Task Generation**: The first LLM will receive the user prompt and generate a task for the subsequent LLM. This task will outline the requirements and specifications for the word document.
-3. **LLM 2: Document Creation**: The second LLM will receive the task generated by the first LLM and create a word document based on the provided specifications.
-&lt;stop_write_ordered_list&gt;
-&lt;write_paragraph&gt;
-## Example Use Case
-&lt;stop_write_paragraph&gt;</t>
+    <t>1. write introduction about Agentic AI
+2. Describe the system architecture
+3. Describe the use cases
+4. Write a conclusion</t>
   </si>
 </sst>
 </file>
@@ -449,7 +439,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="409.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" ht="261" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>2</v>
       </c>

</xml_diff>